<commit_message>
Word export: keep tables as tables, even from crooked photos
- Pages tilted 0.25° or more are straightened before layout analysis.
- Table rules are found where a photo bends them: rows and columns look
  for the rule a little to the side, and line thickness is measured from
  the ink instead of the height a slightly askew rule drifts over. Labels
  in neighbouring merged cells (TOT / USA1 / USA2) no longer run together.
- Small recognition slips are tidied: spaces inside dotted numbers
  ("10.41.22. xx") and a closing bracket missing in a bracketed column.
- The Word review shows tables as tables with merged cells and colours;
  tap a cell to correct it. Lines stay editable fields, and plain-text
  editing is still available.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2KPqXq9Whv7eR2vrvkBWC
</commit_message>
<xml_diff>
--- a/ios/Verification/office-layout/OfficeSampleTable.xlsx
+++ b/ios/Verification/office-layout/OfficeSampleTable.xlsx
@@ -78,7 +78,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFDE6E2"/>
+        <fgColor rgb="FFFBE6E2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -90,7 +90,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8DF71"/>
+        <fgColor rgb="FFF7DE72"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -426,7 +426,7 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.04" customWidth="1"/>
+    <col min="1" max="1" width="8.97" customWidth="1"/>
     <col min="2" max="2" width="22.79" customWidth="1"/>
     <col min="3" max="3" width="1.95" customWidth="1"/>
     <col min="4" max="4" width="30.70" customWidth="1"/>
@@ -454,7 +454,7 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">10.41.22. xx</t>
+          <t xml:space="preserve">10.41.22.xx</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="13.69" customHeight="1">
+    <row r="10" ht="13.91" customHeight="1">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -646,7 +646,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="16.06" customHeight="1">
+    <row r="11" ht="15.84" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">USA1</t>

</xml_diff>